<commit_message>
fix: repair hand-built DCF workbooks so Numbers opens them
scripts/repair_xlsx.py rewrites two defects left by the pre-build-dcf
hand-written workbooks: docProps/core.xml without the Dublin Core
namespace on the root (Numbers rejects the file) and '= label' text
cells stored as formulas. Both rewrites touch only the XML inside the
zip; cell values are unchanged (verified: zero cell diffs against HEAD
on sampled files, --check clean on all 121).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/2CC.NZ/Reports/2CC.NZ_DCF_Model.xlsx
+++ b/research/2CC.NZ/Reports/2CC.NZ_DCF_Model.xlsx
@@ -2458,9 +2458,10 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="3">
-        <f> Reported FCF (Company definition, NZ$M)</f>
-        <v>0</v>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>= Reported FCF (Company definition, NZ$M)</t>
+        </is>
       </c>
       <c r="B8" s="10">
         <v>6.109</v>
@@ -2487,9 +2488,10 @@
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="3">
-        <f> Owner FCF (NZ$M)</f>
-        <v>0</v>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>= Owner FCF (NZ$M)</t>
+        </is>
       </c>
       <c r="B10" s="10">
         <v>4.174</v>
@@ -2516,9 +2518,10 @@
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="3">
-        <f> Owner FCF after SBC (NZ$M)</f>
-        <v>0</v>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>= Owner FCF after SBC (NZ$M)</t>
+        </is>
       </c>
       <c r="B12" s="10">
         <v>4.174</v>

</xml_diff>